<commit_message>
:pen: minor experiment order update
</commit_message>
<xml_diff>
--- a/experiment_blocks.xlsx
+++ b/experiment_blocks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nbaeriswyl\github\VIBE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB86C1E7-19B3-4E62-9132-AB624AAED181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79EE51B-5F33-4AFD-BE23-7E63C21303FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -467,7 +468,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B3">
         <v>15</v>
@@ -493,7 +494,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>20</v>
@@ -731,7 +732,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>15</v>

</xml_diff>

<commit_message>
:sparkles: improve experiment duration
</commit_message>
<xml_diff>
--- a/experiment_blocks.xlsx
+++ b/experiment_blocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nbaeriswyl\github\VIBE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79EE51B-5F33-4AFD-BE23-7E63C21303FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE21DB8E-F421-4008-AD25-20F237F809A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="27">
   <si>
     <t>Session 1</t>
   </si>
@@ -489,7 +488,7 @@
         <v>12</v>
       </c>
       <c r="K3" s="2">
-        <v>8.0000694444444438</v>
+        <v>8.0000925925925923</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -497,7 +496,7 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>11</v>
@@ -515,7 +514,7 @@
         <v>14</v>
       </c>
       <c r="K4" s="2">
-        <v>15.00017361111111</v>
+        <v>15.000231481481482</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -523,7 +522,7 @@
         <v>13</v>
       </c>
       <c r="B5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>11</v>
@@ -532,7 +531,9 @@
       <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" s="1">
+        <v>1</v>
+      </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="J5" t="s">
@@ -547,7 +548,7 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
@@ -556,7 +557,9 @@
         <v>11</v>
       </c>
       <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+      <c r="F6" s="1">
+        <v>1</v>
+      </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="J6" t="s">
@@ -571,7 +574,7 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
@@ -580,8 +583,8 @@
       <c r="E7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>11</v>
+      <c r="F7" s="1">
+        <v>3</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -591,7 +594,7 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
@@ -600,8 +603,8 @@
       <c r="E8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>11</v>
+      <c r="F8" s="1">
+        <v>5</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>11</v>
@@ -616,7 +619,7 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
@@ -650,8 +653,8 @@
         <v>11</v>
       </c>
       <c r="E10" s="1"/>
-      <c r="F10" s="1" t="s">
-        <v>11</v>
+      <c r="F10" s="1">
+        <v>1</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -660,7 +663,7 @@
       </c>
       <c r="K10" s="2">
         <f>K3*SUM(Table1[nb trials])+(COUNT(Table1[nb trials])-1)*K4</f>
-        <v>1845.0164930555554</v>
+        <v>1605.0192129629629</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -675,8 +678,8 @@
       <c r="E11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>11</v>
+      <c r="F11" s="1">
+        <v>3</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
@@ -685,7 +688,7 @@
       </c>
       <c r="K11" s="2">
         <f>SUM(K9:K10)</f>
-        <v>1870.0338541666665</v>
+        <v>1630.036574074074</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -702,8 +705,8 @@
       <c r="E12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>11</v>
+      <c r="F12" s="1">
+        <v>5</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>11</v>
@@ -836,7 +839,7 @@
         <v>12</v>
       </c>
       <c r="K21" s="2">
-        <v>8.0000810185185181</v>
+        <v>8.0001041666666666</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -906,8 +909,8 @@
       <c r="D24" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>11</v>
+      <c r="E24" s="1">
+        <v>3</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>11</v>
@@ -936,8 +939,8 @@
       <c r="D25" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>11</v>
+      <c r="E25" s="1">
+        <v>3</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>11</v>
@@ -1019,7 +1022,7 @@
       </c>
       <c r="K28" s="2">
         <f>K21*SUM(Table2[nb trials])+(COUNT(Table2[nb trials])-1)*K22</f>
-        <v>745.00769675925915</v>
+        <v>745.00954861111109</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -1028,7 +1031,7 @@
       </c>
       <c r="K29" s="2">
         <f>SUM(K27:K28)</f>
-        <v>770.02158564814806</v>
+        <v>770.0234375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
:memo: documentation and experiment tutorial texts
</commit_message>
<xml_diff>
--- a/experiment_blocks.xlsx
+++ b/experiment_blocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nbaeriswyl\github\VIBE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE21DB8E-F421-4008-AD25-20F237F809A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{535768AB-8C19-455F-B4B8-832F9F65134D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="27">
   <si>
     <t>Session 1</t>
   </si>
@@ -630,8 +630,8 @@
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="1" t="s">
-        <v>11</v>
+      <c r="H9" s="1">
+        <v>10</v>
       </c>
       <c r="J9" t="s">
         <v>18</v>
@@ -729,8 +729,8 @@
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="1" t="s">
-        <v>11</v>
+      <c r="H13" s="1">
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>